<commit_message>
Muestreo clínico 16/10: 7 correcciones confirmadas por el autor
</commit_message>
<xml_diff>
--- a/data/revision/revision_20261016.xlsx
+++ b/data/revision/revision_20261016.xlsx
@@ -476,9 +476,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -6823,10 +6821,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/1201430022/1201430022_ft.pdf</t>
         </is>
       </c>
-      <c r="I131" s="5" t="inlineStr"/>
+      <c r="I131" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J131" s="5" t="inlineStr"/>
       <c r="K131" s="5" t="inlineStr"/>
-      <c r="L131" s="5" t="inlineStr"/>
+      <c r="L131" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M131" s="3" t="inlineStr">
         <is>
           <t>regla|aglp1|fuerza|0</t>
@@ -12089,10 +12095,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/67028/67028_ft.pdf</t>
         </is>
       </c>
-      <c r="I241" s="5" t="inlineStr"/>
+      <c r="I241" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J241" s="5" t="inlineStr"/>
       <c r="K241" s="5" t="inlineStr"/>
-      <c r="L241" s="5" t="inlineStr"/>
+      <c r="L241" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M241" s="3" t="inlineStr">
         <is>
           <t>regla|bifosfonatos|equilibrio|0</t>
@@ -15705,10 +15719,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/1211616002/1211616002_ft.pdf</t>
         </is>
       </c>
-      <c r="I317" s="5" t="inlineStr"/>
+      <c r="I317" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J317" s="5" t="inlineStr"/>
       <c r="K317" s="5" t="inlineStr"/>
-      <c r="L317" s="5" t="inlineStr"/>
+      <c r="L317" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M317" s="3" t="inlineStr">
         <is>
           <t>regla|ic_nuevos|general|1</t>
@@ -17511,10 +17533,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/09511001/09511001_ft.pdf</t>
         </is>
       </c>
-      <c r="I355" s="5" t="inlineStr"/>
+      <c r="I355" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J355" s="5" t="inlineStr"/>
       <c r="K355" s="5" t="inlineStr"/>
-      <c r="L355" s="5" t="inlineStr"/>
+      <c r="L355" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M355" s="3" t="inlineStr">
         <is>
           <t>regla|osteoporosis_anabolicos|equilibrio|0</t>
@@ -21280,10 +21310,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/06360001/06360001_ft.pdf</t>
         </is>
       </c>
-      <c r="I434" s="5" t="inlineStr"/>
+      <c r="I434" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J434" s="5" t="inlineStr"/>
       <c r="K434" s="5" t="inlineStr"/>
-      <c r="L434" s="5" t="inlineStr"/>
+      <c r="L434" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M434" s="3" t="inlineStr">
         <is>
           <t>regla|deshabituacion|general|0</t>
@@ -25340,10 +25378,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/61367/61367_ft.pdf</t>
         </is>
       </c>
-      <c r="I518" s="5" t="inlineStr"/>
+      <c r="I518" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J518" s="5" t="inlineStr"/>
       <c r="K518" s="5" t="inlineStr"/>
-      <c r="L518" s="5" t="inlineStr"/>
+      <c r="L518" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M518" s="3" t="inlineStr">
         <is>
           <t>regla|hormonoterapia_prostata|general|0</t>
@@ -31283,10 +31329,18 @@
           <t>https://cima.aemps.es/cima/pdfs/es/ft/62294/62294_ft.pdf</t>
         </is>
       </c>
-      <c r="I643" s="5" t="inlineStr"/>
+      <c r="I643" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="J643" s="5" t="inlineStr"/>
       <c r="K643" s="5" t="inlineStr"/>
-      <c r="L643" s="5" t="inlineStr"/>
+      <c r="L643" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="M643" s="3" t="inlineStr">
         <is>
           <t>regla|antivirales_herpes|general|1</t>
@@ -49364,10 +49418,18 @@
           <t>Evitar. Paracetamol como alternativa. Si se usa ibuprofeno, tomarlo al menos 30 minutos después de la aspirina (o 8 horas antes) para no anular su efecto.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>ddi|3</t>
@@ -55268,10 +55330,18 @@
           <t>No es una contraindicación: su cardiólogo debe conocer la combinación. Tome la nitroglicerina de rescate sentado y levántese despacio.</t>
         </is>
       </c>
-      <c r="F169" s="5" t="inlineStr"/>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="G169" s="5" t="inlineStr"/>
       <c r="H169" s="5" t="inlineStr"/>
-      <c r="I169" s="5" t="inlineStr"/>
+      <c r="I169" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="J169" s="3" t="inlineStr">
         <is>
           <t>ddi|167</t>
@@ -55304,10 +55374,18 @@
           <t>No recomendado por el riesgo de hipotensión sintomática: evitar la combinación.</t>
         </is>
       </c>
-      <c r="F170" s="5" t="inlineStr"/>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
       <c r="G170" s="5" t="inlineStr"/>
       <c r="H170" s="5" t="inlineStr"/>
-      <c r="I170" s="5" t="inlineStr"/>
+      <c r="I170" s="5" t="inlineStr">
+        <is>
+          <t>Confirmado por el autor el 16/10/2026 (muestreo clínico)</t>
+        </is>
+      </c>
       <c r="J170" s="3" t="inlineStr">
         <is>
           <t>ddi|168</t>

</xml_diff>